<commit_message>
chore: 批量初始化 29 个上游 bug issue 处理 plan 并沉淀 issue-plan skill
- 新增 .claude/skills/issue-plan: 为上游 issue 批量生成 plan 与 test-workspace 复现文件的流程规范
- 为 29 个 bug 标签 issue 生成 plan-cweijan-issues-*.md(issue 信息完整摘录+复现数据做实,根因留待分析)
- 复现文件与生成脚本落 test-workspace/(gitignore 内,不入库),登记表见 test-workspace/README.md
- 回填 issues.xlsx 关联 plan 列并刷新 ISSUES.md 快照;agent.md 补充复现文件命名规范引用

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -669,6 +669,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-157-list-nested-table.md</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -789,6 +794,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-204-redo-shortcut-wysiwyg.md</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -829,6 +839,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-218-cmd-h-heading-conflict.md</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -869,6 +884,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-221-csv-copy-paste.md</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -909,6 +929,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-226-kbd-tag-backtick.md</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1069,6 +1094,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-239-large-csv-hang.md</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1229,6 +1259,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-262-paste-image-insiders.md</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1424,6 +1459,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-308-image-rename-variable.md</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1504,6 +1544,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-311-tif-image.md</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1544,6 +1589,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-323-switch-editor-shortcut.md</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1784,6 +1834,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-394-image-upload-path.md</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1824,6 +1879,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-405-image-placeholder.md</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1864,6 +1924,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-415-s3-save-error.md</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1984,6 +2049,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-497-cross-page-table.md</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2064,6 +2134,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-503-wsl-export-chromium.md</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2104,6 +2179,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-529-toc-blank.md</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2184,6 +2264,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-570-scroll-jump-to-top.md</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2224,6 +2309,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-571-codeblock-line-spacing.md</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2264,6 +2354,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-575-table-width-adapt.md</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2304,6 +2399,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-576-sheets-undefined.md</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2504,6 +2604,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-587-local-image-regression.md</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2579,6 +2684,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-590-heading-list-number.md</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2659,6 +2769,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-592-formula-percent-nan.md</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2699,6 +2814,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-593-link-navigation.md</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2819,6 +2939,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-596-md-silent-rewrite.md</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2904,6 +3029,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-598-table-math-formula.md</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2944,6 +3074,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-599-search-result-jump.md</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2984,6 +3119,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-601-trailing-blank-lines.md</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -3062,6 +3202,11 @@
       <c r="G66" t="inlineStr">
         <is>
           <t>待处理</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>docs/plans/plan-cweijan-issues-603-blank-pdf-docx-export.md</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">

</xml_diff>

<commit_message>
chore: 更新 issues.xlsx 处理状态并刷新 ISSUES.md 快照(529/576/592/593)
四个 issue 标记「本项目处理」并附修复摘要备注。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -2176,7 +2176,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2192,6 +2192,11 @@
       <c r="J42" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>已验证被 issue-597 补丁顺带修复(无头渲染 6/6 条目完整),plan 已补全</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2401,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2412,6 +2417,11 @@
       <c r="J47" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>已修复: ExcelJS 加载失败降级 SheetJS 兜底 + 错误面板 i18n,损坏 xlsx 不再崩溃</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2776,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2782,6 +2792,11 @@
       <c r="J56" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>NaN% 主体已由 a97a480(缓存值优先+$分词)修复,本次补 0.0% 小数位语义与保存 round-trip</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2826,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2827,6 +2842,11 @@
       <c r="J57" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>已修复: viewer.js 补 goToDestination/addLinkAttributes,外链经宿主 openExternal 打开</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: 更新 issues.xlsx 处理状态并刷新 ISSUES.md 快照(575/571/590/311/239)
五个 issue 标记「本项目处理」并附修复摘要备注,累计本项目处理 10 个。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1107,6 +1107,11 @@
       <c r="J16" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>已修复: 行数上限 10 万截断+强制只读+横幅提示,CSV 早停/XLSX 体量路由 SheetJS</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1546,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1557,6 +1562,11 @@
       <c r="J27" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>已修复: 新增 tiffMedia 预处理,word 内 TIFF 解码转 PNG 后渲染(utif)</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2321,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2327,6 +2337,11 @@
       <c r="J45" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>已修复: 代码块行高与字号同链(×1.5),修复调大字号后行盒重叠</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2371,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2372,6 +2387,11 @@
       <c r="J46" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>已修复: 移除 vditor 表格单元格 max-width/overflow-wrap 限制,对齐 GFM 表格尺寸语义</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2711,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2707,6 +2727,11 @@
       <c r="J54" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>已修复: 标题转换仅替换所在 li 并保留 data-marker 序号,顺带修多项列表与 IR 模式定位</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: 更新 issues.xlsx 处理状态并刷新 ISSUES.md 快照(497/596/599/601/603)
五个 issue 标记「本项目处理」并附修复摘要备注,累计本项目处理 15 个。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2072,6 +2072,11 @@
       <c r="J39" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>已修复: docx-editor-core patch 追加,跨页表格行不再被切开,整行顺延下页</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2986,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2997,6 +3002,11 @@
       <c r="J60" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>已修复: 保存链路 styleRestore 原文风格还原(diff3),打开零 save 不再 dirty,六类改写消除</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3126,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3132,6 +3142,11 @@
       <c r="J63" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>已修复(缓解): 根因为 VS Code 内核缺口(microsoft/vscode#289785),新增 office.markdown.find 命令经 FindBar 定位</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3176,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3177,6 +3192,11 @@
       <c r="J64" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>已修复: vditor 结尾空行双向保真(trailingBlankLines),round-trip 不再折叠尾部空行</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3266,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3262,6 +3282,11 @@
       <c r="J66" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>已修复: 导出链路异常上抛不再产空白产物误报成功,katex 加载失败降级为原始 LaTeX</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 新增 #295/589/604/607 处理方案,plans 按完成状态归档至 done/todo
- 新增 4 个 issue plan(图片消失/大文件加载慢/嵌套 IF 崩溃/无 dimension 空白)及复现文件生成脚本
- docs/plans 按完成状态整理: 已完成(含修复记录/已修复结论)18 个移入 done/, 待处理 18 个移入 todo/, agent.md 规范留根
- #157/#221 深入分析后确认已修复(随 cweijan-596 及上游提交), 归入 done/
- 同步 issues.xlsx 关联路径、ISSUES.md 快照、test-workspace/README 登记链接与 plan 内相对链接
- 规范同步: agent.md 增加 done/todo 分放规则, issue-plan SKILL 与 sync_issues.py --init 生成路径改为 docs/plans/todo/

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -666,12 +666,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-157-list-nested-table.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-157-list-nested-table.md</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -682,6 +682,11 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-10-05核查:已随cweijan-596(30ae7da styleRestore保存链还原)顺带修复,未编辑区域含表格空行保真;建议实测复现文件收尾</t>
         </is>
       </c>
     </row>
@@ -796,7 +801,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-204-redo-shortcut-wysiwyg.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-204-redo-shortcut-wysiwyg.md</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -807,6 +812,11 @@
       <c r="J9" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-10-05核查:未修复,redo仅匹配Ctrl+Y(editorCommonEvent.ts:264),根因与修复思路已定位见plan</t>
         </is>
       </c>
     </row>
@@ -841,7 +851,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-218-cmd-h-heading-conflict.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-218-cmd-h-heading-conflict.md</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -852,6 +862,11 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-10-05核查:未修复,⌘H hotkey仍在(Options.ts:134)经通用匹配生效,根因与修复思路已定位见plan</t>
         </is>
       </c>
     </row>
@@ -881,12 +896,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>参考cweijan方式完成处理</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-221-csv-copy-paste.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-221-csv-copy-paste.md</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -897,6 +912,11 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-10-05核查:上游c244457(2024-07)已修macOS粘贴,随fork带入;本仓库c9f3279再修mac快捷键;建议实测确认</t>
         </is>
       </c>
     </row>
@@ -931,7 +951,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-226-kbd-tag-backtick.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-226-kbd-tag-backtick.md</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1096,7 +1116,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-239-large-csv-hang.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-239-large-csv-hang.md</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1266,7 +1286,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-262-paste-image-insiders.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-262-paste-image-insiders.md</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1384,6 +1404,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>docs/plans/todo/plan-cweijan-issues-295-image-disappear.md</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -1466,7 +1491,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-308-image-rename-variable.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-308-image-rename-variable.md</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1551,7 +1576,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-311-tif-image.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-311-tif-image.md</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1601,7 +1626,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-323-switch-editor-shortcut.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-323-switch-editor-shortcut.md</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1846,7 +1871,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-394-image-upload-path.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-394-image-upload-path.md</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1891,7 +1916,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-405-image-placeholder.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-405-image-placeholder.md</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1936,7 +1961,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-415-s3-save-error.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-415-s3-save-error.md</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2061,7 +2086,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-497-cross-page-table.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-497-cross-page-table.md</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2151,7 +2176,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-503-wsl-export-chromium.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-503-wsl-export-chromium.md</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2196,7 +2221,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-529-toc-blank.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-529-toc-blank.md</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2286,7 +2311,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-570-scroll-jump-to-top.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-570-scroll-jump-to-top.md</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2331,7 +2356,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-571-codeblock-line-spacing.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-571-codeblock-line-spacing.md</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2381,7 +2406,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-575-table-width-adapt.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-575-table-width-adapt.md</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2431,7 +2456,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-576-sheets-undefined.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-576-sheets-undefined.md</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2641,7 +2666,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-587-local-image-regression.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-587-local-image-regression.md</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2679,6 +2704,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>docs/plans/todo/plan-cweijan-issues-589-large-file-slow-load.md</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -2721,7 +2751,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-590-heading-list-number.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-590-heading-list-number.md</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2811,7 +2841,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-592-formula-percent-nan.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-592-formula-percent-nan.md</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2861,7 +2891,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-593-link-navigation.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-593-link-navigation.md</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -2991,7 +3021,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-596-md-silent-rewrite.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-596-md-silent-rewrite.md</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3036,7 +3066,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-597-word-toc.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-597-word-toc.md</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3086,7 +3116,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-598-table-math-formula.md</t>
+          <t>docs/plans/todo/plan-cweijan-issues-598-table-math-formula.md</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3131,7 +3161,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-599-search-result-jump.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-599-search-result-jump.md</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3181,7 +3211,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-601-trailing-blank-lines.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-601-trailing-blank-lines.md</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3271,7 +3301,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>docs/plans/plan-cweijan-issues-603-blank-pdf-docx-export.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-603-blank-pdf-docx-export.md</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3314,6 +3344,11 @@
           <t>待处理</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>docs/plans/todo/plan-cweijan-issues-604-nested-if-crash.md</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t>2026-09-13 18:33</t>
@@ -3387,6 +3422,11 @@
       <c r="G69" t="inlineStr">
         <is>
           <t>待处理</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>docs/plans/todo/plan-cweijan-issues-607-missing-dimension.md</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">

</xml_diff>

<commit_message>
docs(issues,cweijan-204,cweijan-218): 实测验证通过,plan 归档至 done
验证方式更新为已验证(2026-10-06),xlsx 备注同步,关联路径指向 done/,
并修正 plan 间相对引用(hotkeys-panel/language plan 中 todo/ 指向)。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-204-redo-shortcut-wysiwyg.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-204-redo-shortcut-wysiwyg.md</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-10-05已实施:vditor动作注册表14动作+VSCode命令通道(office.markdown.undo/redo/headings)+vscode-office.markdown.hotkeys设置项,redo默认键补Ctrl+Shift+Z;lint/build通过,待F5实测</t>
+          <t>2026-10-05已实施:动作注册表+VSCode命令通道+hotkeys设置项,redo默认键补Ctrl+Shift+Z;2026-10-06实测验证通过</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-218-cmd-h-heading-conflict.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-218-cmd-h-heading-conflict.md</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-10-05已随cweijan-204实施:headings注册表macOS无默认键不再消费⌘H,可经命令/设置项自定义;待macOS实测(Windows侧Ctrl+H不受影响)</t>
+          <t>2026-10-05已随cweijan-204实施:headings注册表macOS无默认键不再消费⌘H,可经命令/设置项自定义;2026-10-06实测验证通过</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(markdown,cweijan-226): 行内 HTML 标签保存丢失(kbd/mark/span/u/br/img)
Lute 渲染端把行内 HTML 输出为「开标签 span+裸内容+闭标签 span」分离形态,
序列化端只能还原「单 span+完整 data-md-source」形态,往返时标签全部丢失。
在 vditor getMarkdown 序列化前新增 html-inline 规范化重写:栈式由内向外
配对合并为完整标签对,void/自包含形态重写 class 引导单节点还原,残缺
span 退化为字面文本兜底;仅作用于序列化副本,不影响编辑器渲染与交互。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -946,12 +946,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-226-kbd-tag-backtick.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-226-kbd-tag-backtick.md</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -962,6 +962,11 @@
       <c r="J12" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-10-06已实施:vditor序列化前html-inline规范化重写(分离span合并为完整data-md-source),kbd/mark/span/u/br/img等行内HTML保存不再丢标签;F5实测验证通过</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-607): 确认已被 cweijan-576 兜底覆盖无需新修复,plan 归档至 done
同步 issues.xlsx(处理状态→本项目处理、关联 plan 路径、备注补根因结论)
与 ISSUES.md 快照行;test-workspace 登记表本地同步(目录不入库)。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -3426,12 +3426,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-607-missing-dimension.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-607-missing-dimension.md</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3442,6 +3442,11 @@
       <c r="J69" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026-10-06核查:根因为worksheet x:命名空间前缀致ExcelJS抛错,已随cweijan-576 SheetJS兜底覆盖,无代码改动</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-262): 无需处理,plan 归档至 done
2023-09 报告于 VS Code Insiders 每日构建环境(Stable 正常),距今3年该构建已不存在,无法对应现行版本;主线无同类反馈,不跟进

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1286,12 +1286,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-262-paste-image-insiders.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-262-paste-image-insiders.md</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1302,6 +1302,11 @@
       <c r="J20" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-10-06 无需处理:2023-09 报告于 Insiders 每日构建环境(Stable 正常),距今3年该构建已不存在,无法对应现行版本;主线无同类反馈,不跟进</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-295): 无需处理,plan 归档至 done
v3.1.8(2024-02)报告,跨多版本至当前4.x环境无法对应;报告者未跟进录像与细节,触发条件未知;主线无同类反馈,不跟进

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1411,12 +1411,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-295-image-disappear.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-295-image-disappear.md</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1427,6 +1427,11 @@
       <c r="J23" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-10-06 无需处理:v3.1.8(2024-02)报告,跨多版本至当前4.x环境无法对应;报告者未跟进录像与细节,触发条件未知;主线无同类反馈,不跟进</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-308): 实测验证通过,plan 归档至 done
- plan 移入 done/,根因/修复方案/验证方式三节已回填
- issues.xlsx 处理状态改为本项目处理并补核查备注,ISSUES.md 快照同步
- test-workspace 登记表 plan 链接指向 done/(本地文件,不随仓库)

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1501,12 +1501,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-308-image-rename-variable.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-308-image-rename-variable.md</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1517,6 +1517,11 @@
       <c r="J25" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-10-07核查:pasterImgPath 模板变量改为 g 正则+函数替换,重复占位符全量生效,实测通过</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-323): 实测验证通过,plan 归档至 done
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1641,12 +1641,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-323-switch-editor-shortcut.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-323-switch-editor-shortcut.md</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1657,6 +1657,11 @@
       <c r="J28" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-10-07核查:上游5c1072d(宿主keybinding)+378aab8(webview监听)已双通路解决,fork基线已含,现行版本实测通过</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-587): 实测验证通过,plan 归档至 done
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -2686,12 +2686,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-587-local-image-regression.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-587-local-image-regression.md</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2702,6 +2702,11 @@
       <c r="J52" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-10-07核查:根因为 workspacePathAsImageBasePath 开启后相对路径按工作区根解析致落空,配置语义错配非扩展版本回归,无需代码修复,实测验证通过</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-394): 实测验证通过,plan 归档至 done
构造 test-workspace-multi 复现工作区(多仓库父目录布局,已加入 .gitignore),
4.2.2 实测粘贴无 ENOENT,与上游 v4.0.5 已修复的根因结论一致。

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -1891,12 +1891,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-394-image-upload-path.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-394-image-upload-path.md</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1907,6 +1907,11 @@
       <c r="J34" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-10-07核查:上游v4.0.5(ac374ed)已改ensureParentDirectory+vscode.workspace.fs写入,fork基线已含;4.2.2实测父目录工作区粘贴成功无ENOENT,归档</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-604): 实测验证通过,plan 归档至 done
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -3381,12 +3381,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>本项目处理</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-604-nested-if-crash.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-604-nested-if-crash.md</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3397,6 +3397,11 @@
       <c r="J67" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>已修复: renderCell 求值 try/catch 兜底,单格显示 #VALUE!,3层嵌套IF不再导致整文件打开失败(ef61b86)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(issues,cweijan-570): 实测无法复现无需处理,plan 归档至 done
Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/issues/cweijan-issues/issues.xlsx
+++ b/docs/issues/cweijan-issues/issues.xlsx
@@ -2341,12 +2341,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>待处理</t>
+          <t>无需处理</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>docs/plans/todo/plan-cweijan-issues-570-scroll-jump-to-top.md</t>
+          <t>docs/plans/done/plan-cweijan-issues-570-scroll-jump-to-top.md</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2357,6 +2357,11 @@
       <c r="J44" t="inlineStr">
         <is>
           <t>2026-09-13 18:34</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2026-10-08核查:快速输入(含markdown标记字符)实测无法复现跳顶,当前版本无需代码修复,plan内方案A/B保留备查</t>
         </is>
       </c>
     </row>

</xml_diff>